<commit_message>
fix: stageData excel 수정
spawnInterval추가
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/TrainDefenseData.xlsx
+++ b/Assets/02_Resources/Data/TrainDefenseData.xlsx
@@ -1,29 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.4575"/>
-  <workbookPr codeName="ThisWorkbook" autoCompressPictures="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="28545" windowHeight="11700" tabRatio="839" activeTab="5"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" tabRatio="839" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="Monster_Data" sheetId="1" r:id="rId4"/>
-    <sheet name="Train_Data" sheetId="2" r:id="rId5"/>
-    <sheet name="Range_Train_Data" sheetId="3" r:id="rId6"/>
-    <sheet name="Turret_Train_Data" sheetId="4" r:id="rId7"/>
-    <sheet name="Stage_Data" sheetId="5" r:id="rId8"/>
-    <sheet name="Add_Train_Choice_Data" sheetId="6" r:id="rId9"/>
-    <sheet name="Upgrade_Train_Choice_Data" sheetId="7" r:id="rId10"/>
-    <sheet name="Train_Upgrade_Data" sheetId="8" r:id="rId11"/>
-    <sheet name="Turret_Train_Upgrade_Data" sheetId="9" r:id="rId12"/>
-    <sheet name="Range_Train_Upgrade_Data" sheetId="10" r:id="rId13"/>
-    <sheet name="Upgrade_Data" sheetId="11" r:id="rId14"/>
+    <sheet name="Monster_Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Train_Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Range_Train_Data" sheetId="3" r:id="rId3"/>
+    <sheet name="Turret_Train_Data" sheetId="4" r:id="rId4"/>
+    <sheet name="Stage_Data" sheetId="5" r:id="rId5"/>
+    <sheet name="Add_Train_Choice_Data" sheetId="6" r:id="rId6"/>
+    <sheet name="Upgrade_Train_Choice_Data" sheetId="7" r:id="rId7"/>
+    <sheet name="Train_Upgrade_Data" sheetId="8" r:id="rId8"/>
+    <sheet name="Turret_Train_Upgrade_Data" sheetId="9" r:id="rId9"/>
+    <sheet name="Range_Train_Upgrade_Data" sheetId="10" r:id="rId10"/>
+    <sheet name="Upgrade_Data" sheetId="11" r:id="rId11"/>
   </sheets>
+  <calcPr/>
+  <extLst>
+    <ext uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="178">
   <si>
     <t xml:space="preserve">attack_count</t>
   </si>
@@ -265,9 +271,6 @@
     <t xml:space="preserve">1;1;1;</t>
   </si>
   <si>
-    <t xml:space="preserve">180;</t>
-  </si>
-  <si>
     <t xml:space="preserve">포격 포탑</t>
   </si>
   <si>
@@ -557,6 +560,10 @@
   </si>
   <si>
     <t xml:space="preserve">EliteColdAirRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spawn_interval</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -564,7 +571,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -574,31 +581,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
+      <sz val="8"/>
       <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="2">
@@ -610,22 +600,12 @@
     </fill>
   </fills>
   <borders count="12">
-    <border diagonalUp="1" diagonalDown="1">
-      <left>
-        <color indexed="64"/>
-      </left>
-      <right>
-        <color indexed="64"/>
-      </right>
-      <top>
-        <color indexed="64"/>
-      </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -637,12 +617,8 @@
       <top style="medium">
         <color rgb="FF5B9BD5"/>
       </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <bottom/>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -651,15 +627,9 @@
       <right style="medium">
         <color rgb="FF5B9BD5"/>
       </right>
-      <top>
-        <color indexed="64"/>
-      </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -671,12 +641,8 @@
       <top style="medium">
         <color rgb="FFFFC000"/>
       </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <bottom/>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -685,15 +651,9 @@
       <right style="medium">
         <color rgb="FFFFC000"/>
       </right>
-      <top>
-        <color indexed="64"/>
-      </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -702,15 +662,11 @@
       <right style="medium">
         <color rgb="FFFFC000"/>
       </right>
-      <top>
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="medium">
         <color rgb="FFFFC000"/>
       </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -722,12 +678,8 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <bottom/>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -736,15 +688,9 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top>
-        <color indexed="64"/>
-      </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -753,15 +699,11 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top>
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -773,12 +715,8 @@
       <top style="medium">
         <color rgb="FFFFD700"/>
       </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <bottom/>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -787,15 +725,9 @@
       <right style="medium">
         <color rgb="FFFFD700"/>
       </right>
-      <top>
-        <color indexed="64"/>
-      </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
       <left style="medium">
@@ -804,65 +736,19 @@
       <right style="medium">
         <color rgb="FFFFD700"/>
       </right>
-      <top>
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="medium">
         <color rgb="FFFFD700"/>
       </bottom>
-      <diagonal>
-        <color indexed="64"/>
-      </diagonal>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="15">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -938,43 +824,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1000,6 +857,14 @@
           <color rgb="FF8FABDB"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDAE3F3"/>
+          <bgColor rgb="FFDAE3F3"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -1049,72 +914,29 @@
         </right>
       </border>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAE3F3"/>
-          <bgColor rgb="FFDAE3F3"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color rgb="FF8FABDB"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAE3F3"/>
-          <bgColor rgb="FFDAE3F3"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color rgb="FF8FABDB"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAE3F3"/>
-          <bgColor rgb="FFDAE3F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAE3F3"/>
-          <bgColor rgb="FFDAE3F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="1" count="2">
-      <tableStyleElement type="headerRow" size="1" dxfId="1"/>
-      <tableStyleElement type="totalRow" size="1"/>
+    <tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="0" count="1">
+      <tableStyleElement type="headerRow" dxfId="7"/>
     </tableStyle>
-    <tableStyle name="Light Style 1 - Accent 1" pivot="1" table="0" count="7">
-      <tableStyleElement type="wholeTable" size="1" dxfId="2"/>
-      <tableStyleElement type="headerRow" size="1" dxfId="7"/>
-      <tableStyleElement type="totalRow" size="1" dxfId="6"/>
-      <tableStyleElement type="firstColumn" size="1" dxfId="5"/>
-      <tableStyleElement type="lastColumn" size="1" dxfId="5"/>
-      <tableStyleElement type="firstRowStripe" size="1" dxfId="3"/>
-      <tableStyleElement type="firstColumnStripe" size="1" dxfId="4"/>
+    <tableStyle name="Light Style 1 - Accent 1" pivot="0" table="0" count="7">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1161,7 +983,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="2147483647"/>
+        <a:latin typeface="Calibri Light" panose="21474836470000000000"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1213,7 +1035,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="2147483647"/>
+        <a:latin typeface="Calibri" panose="21474836470000000000"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1403,6 +1225,8 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -1410,7 +1234,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:P22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="1" width="9" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.5" style="7" customWidth="1"/>
@@ -1427,7 +1251,7 @@
     <col min="14" max="14" width="13.35546875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
@@ -1435,16 +1259,16 @@
         <v>29</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>34</v>
@@ -1465,21 +1289,21 @@
         <v>26</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A2" s="7">
         <v>10001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D2" s="7">
         <v>10</v>
@@ -1512,10 +1336,10 @@
         <v>73</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A3" s="5">
         <v>10002</v>
       </c>
@@ -1523,7 +1347,7 @@
         <v>76</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D3" s="5">
         <v>35</v>
@@ -1559,12 +1383,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A4" s="5">
         <v>10003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>70</v>
@@ -1600,18 +1424,18 @@
         <v>71</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A5" s="5">
         <v>10004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D5" s="5">
         <v>60</v>
@@ -1644,18 +1468,18 @@
         <v>73</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A6" s="5">
         <v>10005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D6" s="5">
         <v>40</v>
@@ -1688,18 +1512,18 @@
         <v>71</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A7" s="7">
         <v>10006</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D7" s="5">
         <v>200</v>
@@ -1732,15 +1556,15 @@
         <v>73</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A8" s="5">
         <v>10007</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>41</v>
@@ -1776,15 +1600,15 @@
         <v>73</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A9" s="5">
         <v>10008</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>40</v>
@@ -1796,7 +1620,7 @@
         <v>20</v>
       </c>
       <c r="F9" s="7">
-        <v>6.4000000000000004</v>
+        <v>6.4</v>
       </c>
       <c r="G9" s="7">
         <v>1</v>
@@ -1820,18 +1644,18 @@
         <v>73</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A10" s="5">
         <v>10009</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D10" s="5">
         <v>100</v>
@@ -1840,7 +1664,7 @@
         <v>30</v>
       </c>
       <c r="F10" s="7">
-        <v>4.2999999999999998</v>
+        <v>4.3</v>
       </c>
       <c r="G10" s="7">
         <v>1</v>
@@ -1864,15 +1688,15 @@
         <v>73</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A11" s="5">
         <v>10010</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>35</v>
@@ -1908,18 +1732,18 @@
         <v>73</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A12" s="7">
         <v>10011</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D12" s="5">
         <v>30</v>
@@ -1952,10 +1776,10 @@
         <v>73</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A13" s="5">
         <v>10012</v>
       </c>
@@ -1999,12 +1823,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A14" s="5">
         <v>10013</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>74</v>
@@ -2040,18 +1864,18 @@
         <v>73</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A15" s="5">
         <v>10014</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D15" s="5">
         <v>60</v>
@@ -2084,10 +1908,10 @@
         <v>73</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.55">
       <c r="A16" s="5">
         <v>10015</v>
       </c>
@@ -2095,7 +1919,7 @@
         <v>4</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D16" s="5">
         <v>60</v>
@@ -2131,15 +1955,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.55">
       <c r="A17" s="7">
         <v>10016</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D17" s="5">
         <v>300</v>
@@ -2172,18 +1996,18 @@
         <v>73</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.55">
       <c r="A22" s="5">
         <v>10100</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D22" s="5">
         <v>500</v>
@@ -2195,7 +2019,7 @@
         <v>8</v>
       </c>
       <c r="G22" s="7">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="H22" s="7">
         <v>1000</v>
@@ -2216,11 +2040,12 @@
         <v>73</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O22" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -2230,7 +2055,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="15.640625" style="7" customWidth="1"/>
     <col min="3" max="3" width="27.5" style="7" customWidth="1"/>
@@ -2238,7 +2063,7 @@
     <col min="9" max="9" width="19.78515625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
@@ -2246,13 +2071,13 @@
         <v>7</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>26</v>
@@ -2267,15 +2092,15 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A2" s="7">
         <v>100001</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F2" s="7">
         <v>1</v>
@@ -2284,15 +2109,15 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A3" s="7">
         <v>100001</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F3" s="7">
         <v>1</v>
@@ -2301,15 +2126,15 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A4" s="7">
         <v>100001</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F4" s="7">
         <v>1</v>
@@ -2318,15 +2143,15 @@
         <v>250</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A5" s="7">
         <v>100002</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F5" s="7">
         <v>1</v>
@@ -2336,15 +2161,15 @@
       </c>
       <c r="I5" s="8"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A6" s="7">
         <v>100002</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F6" s="7">
         <v>1</v>
@@ -2353,15 +2178,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A7" s="7">
         <v>100002</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F7" s="7">
         <v>1</v>
@@ -2371,6 +2196,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>
@@ -2380,7 +2206,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="27.5703125" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48.5703125" style="7" customWidth="1"/>
@@ -2392,7 +2218,7 @@
     <col min="10" max="10" width="12.140625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
@@ -2400,10 +2226,10 @@
         <v>7</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>13</v>
@@ -2412,17 +2238,17 @@
         <v>59</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>24</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J1" s="8"/>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A2" s="7">
         <v>110001</v>
       </c>
@@ -2430,7 +2256,7 @@
         <v>65</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2448,7 +2274,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A3" s="7">
         <v>110002</v>
       </c>
@@ -2462,7 +2288,7 @@
         <v>200</v>
       </c>
       <c r="E3" s="7">
-        <v>-0.10000000000000001</v>
+        <v>-0.1</v>
       </c>
       <c r="F3" s="7">
         <v>100</v>
@@ -2474,7 +2300,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A4" s="7">
         <v>110003</v>
       </c>
@@ -2482,7 +2308,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D4" s="7">
         <v>50</v>
@@ -2497,18 +2323,18 @@
         <v>3</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A5" s="7">
         <v>110004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D5" s="7">
         <v>300</v>
@@ -2523,15 +2349,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A6" s="7">
         <v>110005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D6" s="7">
         <v>500</v>
@@ -2547,6 +2373,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -2556,42 +2383,42 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="2" width="15.640625" style="7" customWidth="1"/>
     <col min="3" max="3" width="46.28515625" style="7" customWidth="1"/>
     <col min="4" max="13" width="15.640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>17</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A2" s="7">
         <v>20001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>33</v>
@@ -2603,10 +2430,11 @@
         <v>1</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -2616,39 +2444,39 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:M12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="2" width="15.640625" style="7" customWidth="1"/>
     <col min="3" max="3" width="50.28515625" style="7" customWidth="1"/>
     <col min="4" max="5" width="15.640625" style="7" customWidth="1"/>
-    <col min="6" max="6" width="22.65234375" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.640625" style="7" bestFit="1" customWidth="1"/>
     <col min="7" max="10" width="15.640625" style="7" customWidth="1"/>
     <col min="11" max="11" width="18.2109375" style="7" customWidth="1"/>
     <col min="12" max="12" width="21" style="7" customWidth="1"/>
     <col min="13" max="13" width="15.640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>17</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>26</v>
@@ -2663,10 +2491,10 @@
         <v>27</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="16.75">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A2" s="14">
         <v>40001</v>
       </c>
@@ -2674,7 +2502,7 @@
         <v>75</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2701,7 +2529,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A3" s="15">
         <v>40002</v>
       </c>
@@ -2730,28 +2558,28 @@
         <v>1</v>
       </c>
       <c r="K3" s="7">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A4" s="15"/>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A5" s="15"/>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A6" s="15"/>
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="1:12" ht="16.75">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A7" s="21">
         <v>41001</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>18</v>
@@ -2763,7 +2591,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H7" s="7">
         <v>8</v>
@@ -2781,12 +2609,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A8" s="22">
         <v>41002</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>10</v>
@@ -2798,7 +2626,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H8" s="7">
         <v>13</v>
@@ -2810,29 +2638,30 @@
         <v>1</v>
       </c>
       <c r="K8" s="7">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A9" s="22"/>
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A10" s="22"/>
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:2" ht="16.75">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A11" s="23"/>
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>
@@ -2842,7 +2671,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:N21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="1" width="15.640625" style="7" customWidth="1"/>
     <col min="2" max="2" width="17.640625" style="7" customWidth="1"/>
@@ -2854,27 +2683,27 @@
     <col min="12" max="13" width="19.28515625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>17</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>26</v>
@@ -2892,15 +2721,15 @@
         <v>22</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="16.75">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A2" s="9">
         <v>30001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>28</v>
@@ -2933,12 +2762,12 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A3" s="10">
         <v>30002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>61</v>
@@ -2962,16 +2791,16 @@
         <v>1</v>
       </c>
       <c r="K3" s="7">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="L3" s="7">
         <v>0</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A4" s="10">
         <v>30003</v>
       </c>
@@ -2979,7 +2808,7 @@
         <v>77</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D4" s="7">
         <v>100</v>
@@ -3009,15 +2838,15 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A5" s="10">
         <v>30004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D5" s="7">
         <v>100</v>
@@ -3047,15 +2876,15 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A6" s="10">
         <v>30005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D6" s="7">
         <v>100</v>
@@ -3064,7 +2893,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H6" s="7">
         <v>10</v>
@@ -3085,12 +2914,12 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A7" s="10">
         <v>30006</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>68</v>
@@ -3123,15 +2952,15 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A8" s="10">
         <v>30007</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D8" s="7">
         <v>100</v>
@@ -3161,21 +2990,21 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:1">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A9" s="10"/>
     </row>
-    <row r="10" spans="1:1">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A10" s="10"/>
     </row>
-    <row r="11" spans="1:1">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A11" s="10"/>
     </row>
-    <row r="12" spans="1:13" ht="16.75">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A12" s="11">
         <v>31001</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>49</v>
@@ -3187,7 +3016,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H12" s="1">
         <v>10</v>
@@ -3199,7 +3028,7 @@
         <v>1</v>
       </c>
       <c r="K12" s="1">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="L12" s="1">
         <v>0</v>
@@ -3208,12 +3037,12 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A13" s="12">
         <v>31002</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>5</v>
@@ -3225,7 +3054,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H13" s="7">
         <v>10</v>
@@ -3237,21 +3066,21 @@
         <v>1</v>
       </c>
       <c r="K13" s="7">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="L13" s="7">
         <v>0</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="16.75">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A14" s="11">
         <v>31003</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>46</v>
@@ -3263,7 +3092,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H14" s="7">
         <v>10</v>
@@ -3284,12 +3113,12 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A15" s="12">
         <v>31004</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>52</v>
@@ -3301,7 +3130,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H15" s="7">
         <v>10</v>
@@ -3322,12 +3151,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="16.75">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A16" s="11">
         <v>31005</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>8</v>
@@ -3339,7 +3168,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H16" s="7">
         <v>10</v>
@@ -3360,12 +3189,12 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A17" s="12">
         <v>31006</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>19</v>
@@ -3377,7 +3206,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H17" s="7">
         <v>10</v>
@@ -3398,12 +3227,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="16.75">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A18" s="11">
         <v>31007</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>9</v>
@@ -3415,7 +3244,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H18" s="7">
         <v>10</v>
@@ -3436,16 +3265,17 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A19" s="12"/>
     </row>
-    <row r="20" spans="1:1">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A20" s="12"/>
     </row>
-    <row r="21" spans="1:1" ht="16.75">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A21" s="13"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -3454,58 +3284,65 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="1" width="9" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.140625" style="7" customWidth="1"/>
     <col min="3" max="3" width="14.5" style="7" customWidth="1"/>
     <col min="4" max="4" width="23.92578125" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.92578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.78515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.2109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="F1" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A2" s="7">
         <v>50001</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>80</v>
+      <c r="B2" s="7">
+        <v>180</v>
       </c>
       <c r="C2" s="7">
         <v>180</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="E2" s="20" t="s">
         <v>57</v>
-      </c>
-      <c r="E2" s="20" t="s">
-        <v>79</v>
       </c>
       <c r="F2" s="20" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2" s="20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A3" s="2">
         <v>50002</v>
       </c>
@@ -3515,17 +3352,20 @@
       <c r="C3" s="7">
         <v>180</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A4" s="2">
         <v>50003</v>
       </c>
@@ -3535,19 +3375,23 @@
       <c r="C4" s="7">
         <v>180</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>159</v>
+      <c r="D4" s="7">
+        <v>0.5</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>124</v>
+        <v>158</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3555,7 +3399,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="12" style="7" customWidth="1"/>
     <col min="3" max="3" width="12.640625" style="7" customWidth="1"/>
@@ -3565,7 +3409,7 @@
     <col min="7" max="7" width="13.92578125" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
@@ -3573,16 +3417,16 @@
         <v>16</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E1" s="18" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="16.75">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A2" s="14">
         <v>60001</v>
       </c>
@@ -3596,7 +3440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A3" s="15">
         <v>60002</v>
       </c>
@@ -3610,7 +3454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A4" s="15">
         <v>60003</v>
       </c>
@@ -3624,7 +3468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A5" s="15">
         <v>60004</v>
       </c>
@@ -3638,7 +3482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A6" s="15">
         <v>60005</v>
       </c>
@@ -3652,7 +3496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A7" s="15">
         <v>60006</v>
       </c>
@@ -3666,7 +3510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A8" s="15">
         <v>60007</v>
       </c>
@@ -3680,7 +3524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A9" s="15">
         <v>60008</v>
       </c>
@@ -3694,7 +3538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A10" s="15">
         <v>60009</v>
       </c>
@@ -3708,43 +3552,43 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A11" s="15"/>
       <c r="D11" s="19">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A12" s="15"/>
       <c r="D12" s="19">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A13" s="15"/>
       <c r="D13" s="19">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A14" s="15"/>
       <c r="D14" s="19">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A15" s="15"/>
       <c r="D15" s="19">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="16.75">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A16" s="16"/>
       <c r="D16" s="19">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A17" s="6">
         <v>61001</v>
       </c>
@@ -3759,6 +3603,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -3768,7 +3613,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="1" width="10" style="6" customWidth="1"/>
     <col min="2" max="2" width="13.92578125" style="7" customWidth="1"/>
@@ -3777,7 +3622,7 @@
     <col min="5" max="5" width="13.78515625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
@@ -3788,13 +3633,13 @@
         <v>62</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="16.75">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A2" s="14">
         <v>70001</v>
       </c>
@@ -3811,7 +3656,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A3" s="15">
         <v>70002</v>
       </c>
@@ -3828,7 +3673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A4" s="15">
         <v>70003</v>
       </c>
@@ -3845,7 +3690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A5" s="15">
         <v>70004</v>
       </c>
@@ -3862,7 +3707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A6" s="15">
         <v>70005</v>
       </c>
@@ -3879,7 +3724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A7" s="15">
         <v>70006</v>
       </c>
@@ -3896,7 +3741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A8" s="15">
         <v>70007</v>
       </c>
@@ -3913,7 +3758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A9" s="15">
         <v>70008</v>
       </c>
@@ -3930,7 +3775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A10" s="15">
         <v>70009</v>
       </c>
@@ -3947,40 +3792,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:1">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A11" s="15"/>
     </row>
-    <row r="12" spans="1:1">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A12" s="15"/>
     </row>
-    <row r="13" spans="1:1">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A13" s="15"/>
     </row>
-    <row r="14" spans="1:1">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A14" s="15"/>
     </row>
-    <row r="15" spans="1:1">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A15" s="15"/>
     </row>
-    <row r="16" spans="1:1" ht="16.75">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A16" s="16"/>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.55">
       <c r="A17" s="17"/>
     </row>
-    <row r="18" spans="1:1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.55">
       <c r="A18" s="17"/>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.55">
       <c r="A19" s="17"/>
     </row>
-    <row r="20" spans="1:1">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.55">
       <c r="A20" s="17"/>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.55">
       <c r="A21" s="17"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>
@@ -3990,13 +3836,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="1" width="15.78515625" style="7" customWidth="1"/>
     <col min="2" max="2" width="13.5" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
@@ -4004,21 +3850,22 @@
         <v>7</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A2" s="7">
         <v>80001</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -4028,7 +3875,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:J22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="17.28515625" style="7" customWidth="1"/>
     <col min="3" max="3" width="35.0703125" style="7" customWidth="1"/>
@@ -4040,7 +3887,7 @@
     <col min="9" max="9" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
@@ -4048,13 +3895,13 @@
         <v>7</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>26</v>
@@ -4069,15 +3916,15 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A2" s="7">
         <v>90001</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G2" s="7">
         <v>5</v>
@@ -4086,15 +3933,15 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A3" s="7">
         <v>90001</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G3" s="7">
         <v>10</v>
@@ -4103,15 +3950,15 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A4" s="7">
         <v>90001</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G4" s="7">
         <v>25</v>
@@ -4120,150 +3967,150 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A5" s="7">
         <v>90002</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G5" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A6" s="7">
         <v>90002</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G6" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A7" s="7">
         <v>90002</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G7" s="7">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A8" s="7">
         <v>90003</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G8" s="7">
         <v>15</v>
       </c>
       <c r="I8" s="7">
-        <v>0.14999999999999999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A9" s="7">
         <v>90003</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G9" s="7">
         <v>20</v>
       </c>
       <c r="I9" s="7">
-        <v>0.14999999999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A10" s="7">
         <v>90003</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G10" s="7">
         <v>40</v>
       </c>
       <c r="I10" s="7">
-        <v>0.20000000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A11" s="6">
         <v>90004</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G11" s="7">
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A12" s="7">
         <v>90004</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G12" s="7">
         <v>150</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A13" s="7">
         <v>90004</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G13" s="7">
         <v>250</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A14" s="6">
         <v>90005</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G14" s="7">
         <v>3</v>
@@ -4272,15 +4119,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A15" s="7">
         <v>90005</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G15" s="7">
         <v>5</v>
@@ -4289,15 +4136,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A16" s="7">
         <v>90005</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G16" s="7">
         <v>7</v>
@@ -4306,15 +4153,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A17" s="6">
         <v>90006</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F17" s="7">
         <v>1</v>
@@ -4323,15 +4170,15 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A18" s="7">
         <v>90006</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F18" s="7">
         <v>1</v>
@@ -4340,15 +4187,15 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A19" s="8">
         <v>90006</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F19" s="7">
         <v>1</v>
@@ -4357,49 +4204,50 @@
         <v>200</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A20" s="8">
         <v>90007</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G20" s="7">
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A21" s="8">
         <v>90007</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G21" s="7">
         <v>150</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A22" s="8">
         <v>90007</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G22" s="7">
         <v>350</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699722230434418" right="0.699722230434418" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
fix : 이미지 변경과 애니메이션 적용 ElectrickProjectile, LaserProjectile , 코드 수정 ApplyScaleByAttackRange
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/TrainDefenseData.xlsx
+++ b/Assets/02_Resources/Data/TrainDefenseData.xlsx
@@ -25,202 +25,382 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="178">
   <si>
+    <t xml:space="preserve">weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">damage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">폭발 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_hp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">해골 병사다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1;1;1;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미노타우로스다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레이저 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dwarf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">해골 왕이당.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lizard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">icon_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고블린 거인</t>
+  </si>
+  <si>
+    <t xml:space="preserve">도마뱀이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거북이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">놀이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxHp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ranged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">상어다 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turtle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skull</t>
+  </si>
+  <si>
+    <t xml:space="preserve">난쟁이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gnoll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spider</t>
+  </si>
+  <si>
+    <t xml:space="preserve">냉기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">메인 기차</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">도적이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">귀상어다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">판다다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">곰이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">뱀이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거미다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteLaserTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FireEffectProjectile</t>
+  </si>
+  <si>
     <t xml:space="preserve">EliteColdAirRangeTrain</t>
   </si>
   <si>
+    <t xml:space="preserve">레이저로 강하게 지속적인 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteNormalTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteCannonTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 공격 범위 {1} 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElectrickTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spawn_monsters_level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteFireTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 공격딜레이 {1} 감소</t>
+  </si>
+  <si>
+    <t xml:space="preserve">획득하는 경험치 {0}/{1} % 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 범위 {1} 증가</t>
+  </si>
+  <si>
     <t xml:space="preserve">EliteMissileTurretTrain</t>
   </si>
   <si>
+    <t xml:space="preserve">EliteSniperTurretTrain</t>
+  </si>
+  <si>
     <t xml:space="preserve">획득하는 골드 {0}/{1} % 증가</t>
   </si>
   <si>
+    <t xml:space="preserve">projectile_prefab_id</t>
+  </si>
+  <si>
     <t xml:space="preserve">stage_inspection_time</t>
   </si>
   <si>
-    <t xml:space="preserve">ElectrickTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteCannonTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteLaserTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteNormalTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저로 강하게 지속적인 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 공격 범위 {1} 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">획득하는 경험치 {0}/{1} % 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">projectile_prefab_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FireEffectProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 범위 {1} 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spawn_monsters_level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteSniperTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteFireTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 공격딜레이 {1} 감소</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거미다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">판다다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">곰이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">뱀이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ranged</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thief</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미노타우로스다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폭발 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">놀이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">냉기 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spider</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Melee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">도적이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Snake</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">해골 병사다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">메인 기차</t>
-  </si>
-  <si>
-    <t xml:space="preserve">난쟁이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gnoll</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">귀상어다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1;1;1;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lizard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">상어다 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">해골 왕이당.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Turtle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">도마뱀이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dwarf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxHp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고블린 거인</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거북이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_hp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skull</t>
-  </si>
-  <si>
-    <t xml:space="preserve">icon_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">damage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shark</t>
+    <t xml:space="preserve">공격력 {0}/{1} % 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MissileProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ColdAirProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SniperProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10004;10005;10006;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레이저 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MissileTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">replace_train_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10001;10002;10003;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염으로 지속적인 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NormalTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SniperTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CannonProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격 딜레이 {0}/{1} % 감소</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NormalProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LaserTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExplosionRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weighted_upgrades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_upgrade_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExplosionProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ColdAirRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CannonTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElectrickProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 기관총 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">train_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">폭발 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 전기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hammershark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GiantGoblin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전기 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 폭발 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MainTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고블린 주술사다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">냉기 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minotaur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SkullKing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포격 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prefab_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 포격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 미사일 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 냉기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">move_speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stat_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GoblinSpear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 레이저 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">need_money</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레이저 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1;1;1;1;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 저격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고블린 창병이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 화염 포탑</t>
   </si>
   <si>
     <t xml:space="preserve">포탑들의 공격 딜레이가 {0}({1})만큼 감소합니다.</t>
@@ -238,325 +418,145 @@
     <t xml:space="preserve">적 처치 시 획득하는 골드가 {0}({1})만큼 증가합니다.</t>
   </si>
   <si>
-    <t xml:space="preserve">엘리트 기관총 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 전기 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">train_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 폭발 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SkullKing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고블린 주술사다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폭발 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hammershark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stat_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MainTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 화염 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GoblinSpear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 냉기 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GiantGoblin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">냉기 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minotaur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 레이저 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">move_speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고블린 창병이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1;1;1;1;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">need_money</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 포격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 저격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prefab_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 미사일 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MissileTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CannonTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SniperTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">replace_train_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격 딜레이 {0}/{1} % 감소</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SniperProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10001;10002;10003;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElectrickProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_upgrade_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LaserTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExplosionProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NormalTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExplosionRangeTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CannonProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MissileProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">weighted_upgrades</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ColdAirRangeTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NormalProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0}/{1} % 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10004;10005;10006;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염으로 지속적인 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ColdAirProjectile</t>
+    <t xml:space="preserve">drop_money_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonTrainUpgrade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">체력 {0}/{1} % 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총으로 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TrainUpgrade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_exp_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AttackDamage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GoblinSorcerer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AttackInterval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포격 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">폭발 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">train_data_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">제일 기본이 되는 기차이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LaserProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_delay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FireTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_exp_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spawn_monsters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">냉기 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_damage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_money_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target_train_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stage_end_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_main_train</t>
+  </si>
+  <si>
+    <t xml:space="preserve">monster_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_interval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spawn_interval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전기 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10007;10008;10009;10010;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포탑들의 공격력이 {0}({1})만큼 증가합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteExplosionRangeTrain</t>
   </si>
   <si>
     <t xml:space="preserve">저격을 발사해 몇 초 후 강한 피해를 준다.</t>
   </si>
   <si>
+    <t xml:space="preserve">범위 내에 있는 적들을 밀치고 피해를 준다.</t>
+  </si>
+  <si>
     <t xml:space="preserve">미사일로 강한 피해를 준다. 공격속도는 느리다.</t>
   </si>
   <si>
-    <t xml:space="preserve">EliteExplosionRangeTrain</t>
+    <t xml:space="preserve">spawn_monsters_probability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 공격하는 적 수 {1} 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화면에 있는 다수의 적들을 전기로 공격한다.</t>
   </si>
   <si>
     <t xml:space="preserve">포탑들의 체력이 {0}({1})만큼 증가합니다.</t>
   </si>
   <si>
-    <t xml:space="preserve">공격력 {0} 증가 공격하는 적 수 {1} 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spawn_monsters_probability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화면에 있는 다수의 적들을 전기로 공격한다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">범위 내에 있는 적들을 밀치고 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포탑들의 공격력이 {0}({1})만큼 증가합니다.</t>
-  </si>
-  <si>
     <t xml:space="preserve">EliteElectrickTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10007;10008;10009;10010;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GoblinSorcerer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">체력 {0}/{1} % 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonTrainUpgrade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TrainUpgrade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">train_data_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">target_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AttackDamage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AttackInterval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_money_min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총으로 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_damage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폭발 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_exp_min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_interval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stage_end_time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">monster_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_exp_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LaserProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_money_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">냉기 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spawn_monsters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">is_main_train</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FireTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">target_train_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">제일 기본이 되는 기차이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_delay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spawn_interval</t>
   </si>
 </sst>
 </file>
@@ -945,28 +945,7 @@
   <cellStyles count="1">
     <cellStyle xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAE3F3"/>
-          <bgColor rgb="FFDAE3F3"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color rgb="FF8FABDB"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAE3F3"/>
-          <bgColor rgb="FFDAE3F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1092,15 +1071,13 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="1" count="1">
-      <tableStyleElement type="headerRow" size="1" dxfId="6"/>
+      <tableStyleElement type="headerRow" size="1" dxfId="4"/>
     </tableStyle>
-    <tableStyle name="Light Style 1 - Accent 1" pivot="0" table="1" count="6">
-      <tableStyleElement type="wholeTable" size="1" dxfId="5"/>
-      <tableStyleElement type="headerRow" size="1" dxfId="4"/>
-      <tableStyleElement type="totalRow" size="1" dxfId="3"/>
-      <tableStyleElement type="firstColumn" size="1" dxfId="2"/>
-      <tableStyleElement type="lastColumn" size="1" dxfId="1"/>
-      <tableStyleElement type="firstRowStripe" size="1"/>
+    <tableStyle name="Light Style 1 - Accent 1" pivot="0" table="1" count="4">
+      <tableStyleElement type="wholeTable" size="1" dxfId="3"/>
+      <tableStyleElement type="headerRow" size="1" dxfId="2"/>
+      <tableStyleElement type="totalRow" size="1" dxfId="1"/>
+      <tableStyleElement type="firstColumn" size="1"/>
     </tableStyle>
   </tableStyles>
 </styleSheet>
@@ -1417,46 +1394,46 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>176</v>
+        <v>151</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -1464,10 +1441,10 @@
         <v>10001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="D2" s="7">
         <v>10</v>
@@ -1479,16 +1456,16 @@
         <v>5</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="I2" s="7">
         <v>10</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="K2" s="7">
         <v>10</v>
@@ -1497,10 +1474,10 @@
         <v>2</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -1508,10 +1485,10 @@
         <v>10002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D3" s="5">
         <v>35</v>
@@ -1541,10 +1518,10 @@
         <v>1.5</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -1552,10 +1529,10 @@
         <v>10003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="D4" s="5">
         <v>50</v>
@@ -1588,7 +1565,7 @@
         <v>25</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -1596,10 +1573,10 @@
         <v>10004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D5" s="5">
         <v>60</v>
@@ -1629,10 +1606,10 @@
         <v>2</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -1640,10 +1617,10 @@
         <v>10005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="D6" s="5">
         <v>40</v>
@@ -1676,7 +1653,7 @@
         <v>25</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>65</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -1684,10 +1661,10 @@
         <v>10006</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="D7" s="5">
         <v>200</v>
@@ -1717,10 +1694,10 @@
         <v>2</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -1728,10 +1705,10 @@
         <v>10007</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="D8" s="5">
         <v>40</v>
@@ -1761,10 +1738,10 @@
         <v>3</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -1772,10 +1749,10 @@
         <v>10008</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="D9" s="5">
         <v>70</v>
@@ -1805,10 +1782,10 @@
         <v>1.5</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -1816,10 +1793,10 @@
         <v>10009</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="D10" s="5">
         <v>100</v>
@@ -1849,10 +1826,10 @@
         <v>1.5</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>48</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -1860,10 +1837,10 @@
         <v>10010</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D11" s="5">
         <v>150</v>
@@ -1893,10 +1870,10 @@
         <v>2</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -1904,10 +1881,10 @@
         <v>10011</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D12" s="5">
         <v>30</v>
@@ -1937,10 +1914,10 @@
         <v>2</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -1951,7 +1928,7 @@
         <v>32</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="D13" s="5">
         <v>100</v>
@@ -1981,7 +1958,7 @@
         <v>3</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N13" s="2" t="s">
         <v>32</v>
@@ -1992,10 +1969,10 @@
         <v>10013</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D14" s="5">
         <v>250</v>
@@ -2025,10 +2002,10 @@
         <v>2</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -2036,10 +2013,10 @@
         <v>10014</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
       <c r="D15" s="5">
         <v>60</v>
@@ -2069,10 +2046,10 @@
         <v>2</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -2083,7 +2060,7 @@
         <v>142</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="D16" s="5">
         <v>60</v>
@@ -2124,10 +2101,10 @@
         <v>10016</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="D17" s="5">
         <v>300</v>
@@ -2157,10 +2134,10 @@
         <v>2</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -2168,10 +2145,10 @@
         <v>10100</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>79</v>
+        <v>108</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D22" s="5">
         <v>500</v>
@@ -2201,10 +2178,10 @@
         <v>3</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>79</v>
+        <v>108</v>
       </c>
       <c r="O22" s="2"/>
     </row>
@@ -2228,31 +2205,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>156</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -2260,10 +2237,10 @@
         <v>100001</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="F2" s="7">
         <v>1</v>
@@ -2277,10 +2254,10 @@
         <v>100001</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="F3" s="7">
         <v>1</v>
@@ -2294,10 +2271,10 @@
         <v>100001</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="F4" s="7">
         <v>1</v>
@@ -2311,10 +2288,10 @@
         <v>100002</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="F5" s="7">
         <v>1</v>
@@ -2329,10 +2306,10 @@
         <v>100002</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="F6" s="7">
         <v>1</v>
@@ -2346,10 +2323,10 @@
         <v>100002</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="F7" s="7">
         <v>1</v>
@@ -2382,31 +2359,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F1" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>115</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>84</v>
       </c>
       <c r="J1" s="8"/>
     </row>
@@ -2415,10 +2392,10 @@
         <v>110001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>127</v>
+        <v>66</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>139</v>
+        <v>168</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2430,10 +2407,10 @@
         <v>100</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2441,10 +2418,10 @@
         <v>110002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>111</v>
+        <v>80</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="D3" s="7">
         <v>200</v>
@@ -2456,10 +2433,10 @@
         <v>100</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2467,10 +2444,10 @@
         <v>110003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>134</v>
+        <v>176</v>
       </c>
       <c r="D4" s="7">
         <v>50</v>
@@ -2482,10 +2459,10 @@
         <v>50</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2493,10 +2470,10 @@
         <v>110004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="D5" s="7">
         <v>300</v>
@@ -2508,7 +2485,7 @@
         <v>10</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2516,10 +2493,10 @@
         <v>110005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>69</v>
+        <v>129</v>
       </c>
       <c r="D6" s="7">
         <v>500</v>
@@ -2531,7 +2508,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2553,25 +2530,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2579,10 +2556,10 @@
         <v>20001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>175</v>
+        <v>149</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2591,7 +2568,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2618,40 +2595,40 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>156</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2659,10 +2636,10 @@
         <v>40001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2671,7 +2648,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>120</v>
+        <v>84</v>
       </c>
       <c r="H2" s="7">
         <v>5</v>
@@ -2686,7 +2663,7 @@
         <v>4</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>118</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -2694,10 +2671,10 @@
         <v>40002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>68</v>
+        <v>128</v>
       </c>
       <c r="D3" s="7">
         <v>100</v>
@@ -2706,7 +2683,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>125</v>
+        <v>88</v>
       </c>
       <c r="H3" s="7">
         <v>5</v>
@@ -2721,7 +2698,7 @@
         <v>0.10000000000000001</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>130</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:1">
@@ -2739,10 +2716,10 @@
         <v>41001</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="D7" s="7">
         <v>150</v>
@@ -2751,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>133</v>
+        <v>169</v>
       </c>
       <c r="H7" s="7">
         <v>8</v>
@@ -2766,7 +2743,7 @@
         <v>4</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>118</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2774,10 +2751,10 @@
         <v>41002</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="D8" s="7">
         <v>150</v>
@@ -2786,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H8" s="7">
         <v>13</v>
@@ -2801,7 +2778,7 @@
         <v>0.10000000000000001</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>130</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2844,43 +2821,43 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>156</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -2888,10 +2865,10 @@
         <v>30001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2900,7 +2877,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>119</v>
+        <v>76</v>
       </c>
       <c r="H2" s="7">
         <v>10</v>
@@ -2918,7 +2895,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="8" t="s">
-        <v>126</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2926,10 +2903,10 @@
         <v>30002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="D3" s="7">
         <v>100</v>
@@ -2938,7 +2915,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>172</v>
+        <v>152</v>
       </c>
       <c r="H3" s="7">
         <v>10</v>
@@ -2956,7 +2933,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2964,10 +2941,10 @@
         <v>30003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>132</v>
+        <v>172</v>
       </c>
       <c r="D4" s="7">
         <v>100</v>
@@ -2976,7 +2953,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="H4" s="7">
         <v>10</v>
@@ -2994,7 +2971,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>123</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -3002,10 +2979,10 @@
         <v>30004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="D5" s="7">
         <v>100</v>
@@ -3014,7 +2991,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>117</v>
+        <v>82</v>
       </c>
       <c r="H5" s="7">
         <v>15</v>
@@ -3032,7 +3009,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3040,10 +3017,10 @@
         <v>30005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>63</v>
+        <v>9</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>137</v>
+        <v>175</v>
       </c>
       <c r="D6" s="7">
         <v>100</v>
@@ -3052,7 +3029,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="H6" s="7">
         <v>10</v>
@@ -3070,7 +3047,7 @@
         <v>5</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3078,10 +3055,10 @@
         <v>30006</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>67</v>
+        <v>127</v>
       </c>
       <c r="D7" s="7">
         <v>100</v>
@@ -3090,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="H7" s="7">
         <v>10</v>
@@ -3108,7 +3085,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -3116,10 +3093,10 @@
         <v>30007</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>131</v>
+        <v>170</v>
       </c>
       <c r="D8" s="7">
         <v>100</v>
@@ -3128,7 +3105,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="H8" s="7">
         <v>10</v>
@@ -3146,7 +3123,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>112</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:1">
@@ -3163,10 +3140,10 @@
         <v>31001</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>122</v>
+        <v>77</v>
       </c>
       <c r="D12" s="7">
         <v>150</v>
@@ -3175,7 +3152,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="H12" s="1">
         <v>10</v>
@@ -3193,7 +3170,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="8" t="s">
-        <v>126</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -3201,10 +3178,10 @@
         <v>31002</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="D13" s="7">
         <v>150</v>
@@ -3213,7 +3190,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="H13" s="7">
         <v>10</v>
@@ -3231,7 +3208,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -3239,10 +3216,10 @@
         <v>31003</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>116</v>
+        <v>83</v>
       </c>
       <c r="D14" s="7">
         <v>150</v>
@@ -3251,7 +3228,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>1</v>
+        <v>61</v>
       </c>
       <c r="H14" s="7">
         <v>10</v>
@@ -3269,7 +3246,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>123</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -3277,10 +3254,10 @@
         <v>31004</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>107</v>
+        <v>71</v>
       </c>
       <c r="D15" s="7">
         <v>150</v>
@@ -3289,7 +3266,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="H15" s="7">
         <v>10</v>
@@ -3307,7 +3284,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -3315,10 +3292,10 @@
         <v>31005</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D16" s="7">
         <v>150</v>
@@ -3327,7 +3304,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>140</v>
+        <v>177</v>
       </c>
       <c r="H16" s="7">
         <v>10</v>
@@ -3345,7 +3322,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -3353,10 +3330,10 @@
         <v>31006</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="D17" s="7">
         <v>150</v>
@@ -3365,7 +3342,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="H17" s="7">
         <v>10</v>
@@ -3383,7 +3360,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -3391,10 +3368,10 @@
         <v>31007</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="D18" s="7">
         <v>150</v>
@@ -3403,7 +3380,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="H18" s="7">
         <v>10</v>
@@ -3421,7 +3398,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>112</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -3456,25 +3433,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>3</v>
+        <v>65</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>136</v>
+        <v>173</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3491,13 +3468,13 @@
         <v>0.5</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -3514,13 +3491,13 @@
         <v>0.5</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -3537,13 +3514,13 @@
         <v>0.5</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>141</v>
+        <v>167</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -3568,19 +3545,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>110</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="16.75">
@@ -3619,7 +3596,7 @@
         <v>30003</v>
       </c>
       <c r="C4" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="19">
         <v>0</v>
@@ -3647,7 +3624,7 @@
         <v>30005</v>
       </c>
       <c r="C6" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="19">
         <v>0</v>
@@ -3780,19 +3757,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>124</v>
+        <v>85</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.75">
@@ -3999,19 +3976,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -4043,31 +4020,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>156</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -4075,10 +4052,10 @@
         <v>90001</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="G2" s="7">
         <v>5</v>
@@ -4092,10 +4069,10 @@
         <v>90001</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="G3" s="7">
         <v>10</v>
@@ -4109,10 +4086,10 @@
         <v>90001</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="G4" s="7">
         <v>25</v>
@@ -4126,7 +4103,7 @@
         <v>90002</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>94</v>
@@ -4140,7 +4117,7 @@
         <v>90002</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>94</v>
@@ -4154,7 +4131,7 @@
         <v>90002</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>94</v>
@@ -4168,10 +4145,10 @@
         <v>90003</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="G8" s="7">
         <v>15</v>
@@ -4185,10 +4162,10 @@
         <v>90003</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="G9" s="7">
         <v>20</v>
@@ -4202,10 +4179,10 @@
         <v>90003</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="G10" s="7">
         <v>40</v>
@@ -4219,7 +4196,7 @@
         <v>90004</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>94</v>
@@ -4233,7 +4210,7 @@
         <v>90004</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>94</v>
@@ -4247,7 +4224,7 @@
         <v>90004</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>94</v>
@@ -4261,10 +4238,10 @@
         <v>90005</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="G14" s="7">
         <v>3</v>
@@ -4278,10 +4255,10 @@
         <v>90005</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="G15" s="7">
         <v>5</v>
@@ -4295,10 +4272,10 @@
         <v>90005</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="G16" s="7">
         <v>7</v>
@@ -4312,10 +4289,10 @@
         <v>90006</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>9</v>
+        <v>54</v>
       </c>
       <c r="F17" s="7">
         <v>1</v>
@@ -4329,10 +4306,10 @@
         <v>90006</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>9</v>
+        <v>54</v>
       </c>
       <c r="F18" s="7">
         <v>1</v>
@@ -4346,10 +4323,10 @@
         <v>90006</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>9</v>
+        <v>54</v>
       </c>
       <c r="F19" s="7">
         <v>1</v>
@@ -4363,7 +4340,7 @@
         <v>90007</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>94</v>
@@ -4377,7 +4354,7 @@
         <v>90007</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>94</v>
@@ -4391,7 +4368,7 @@
         <v>90007</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>94</v>

</xml_diff>

<commit_message>
fix : Projectile이 사라질 때 TriggerHandle을 생성하도록 수정
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/TrainDefenseData.xlsx
+++ b/Assets/02_Resources/Data/TrainDefenseData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.4575"/>
   <workbookPr codeName="ThisWorkbook" autoCompressPictures="1"/>
   <bookViews>
-    <workbookView windowWidth="28545" windowHeight="11700" tabRatio="839" activeTab="5"/>
+    <workbookView windowWidth="28545" windowHeight="11700" tabRatio="839" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Monster_Data" sheetId="1" r:id="rId4"/>
@@ -23,519 +23,531 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="179">
+  <si>
+    <t xml:space="preserve">spawn_monsters_level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 범위 {1} 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">획득하는 경험치 {0}/{1} % 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FireEffectProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteCannonTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteLaserTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 공격딜레이 {1} 감소</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteSniperTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레이저로 강하게 지속적인 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">projectile_prefab_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteMissileTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stage_inspection_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteNormalTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 공격 범위 {1} 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">획득하는 골드 {0}/{1} % 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteFireTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteColdAirRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElectrickTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">곰이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거미다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">뱀이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">판다다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10004;10005;10006;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CannonTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_upgrade_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElectrickProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SniperTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExplosionProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weighted_upgrades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MissileProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ColdAirProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LaserTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExplosionRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NormalProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염으로 지속적인 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0}/{1} % 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CannonProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10001;10002;10003;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레이저 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격 딜레이 {0}/{1} % 감소</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ColdAirRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MissileTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SniperProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NormalTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">replace_train_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">폭발 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonTrainUpgrade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">체력 {0}/{1} % 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총으로 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포격 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AttackDamage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전기 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_delay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AttackInterval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_exp_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FireTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GoblinSorcerer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">monster_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TrainUpgrade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">냉기 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_main_train</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stage_end_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_money_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LaserProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spawn_monsters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_money_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target_train_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_interval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">train_data_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">제일 기본이 되는 기차이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_exp_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_damage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spawn_interval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포탑들의 공격 딜레이가 {0}({1})만큼 감소합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">범위 내에 있는 적들의 이동속도가 느려지고 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거대한 미사일을 발사해 몇 초 후 광역 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">메인 기차</t>
+  </si>
+  <si>
+    <t xml:space="preserve">도적이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레이저 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">damage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">해골 병사다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미노타우로스다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dwarf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1;1;1;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고블린 거인</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxHp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">폭발 포탑</t>
+  </si>
   <si>
     <t xml:space="preserve">weight</t>
   </si>
   <si>
-    <t xml:space="preserve">damage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폭발 포탑</t>
+    <t xml:space="preserve">Turtle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">놀이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거북이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lizard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">도마뱀이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">난쟁이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">상어다 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skull</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gnoll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">냉기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">해골 왕이당.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ranged</t>
   </si>
   <si>
     <t xml:space="preserve">max_hp</t>
   </si>
   <si>
-    <t xml:space="preserve">해골 병사다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1;1;1;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미노타우로스다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dwarf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thief</t>
-  </si>
-  <si>
-    <t xml:space="preserve">해골 왕이당.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lizard</t>
-  </si>
-  <si>
     <t xml:space="preserve">icon_id</t>
   </si>
   <si>
-    <t xml:space="preserve">Panda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고블린 거인</t>
-  </si>
-  <si>
-    <t xml:space="preserve">도마뱀이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거북이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">놀이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxHp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ranged</t>
-  </si>
-  <si>
-    <t xml:space="preserve">상어다 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Turtle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skull</t>
-  </si>
-  <si>
-    <t xml:space="preserve">난쟁이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gnoll</t>
+    <t xml:space="preserve">귀상어다.</t>
   </si>
   <si>
     <t xml:space="preserve">Spider</t>
   </si>
   <si>
-    <t xml:space="preserve">냉기 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Snake</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">메인 기차</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Melee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">도적이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">귀상어다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">판다다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">곰이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">뱀이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거미다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteLaserTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FireEffectProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteColdAirRangeTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저로 강하게 지속적인 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteNormalTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteCannonTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 공격 범위 {1} 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElectrickTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spawn_monsters_level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteFireTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 공격딜레이 {1} 감소</t>
-  </si>
-  <si>
-    <t xml:space="preserve">획득하는 경험치 {0}/{1} % 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 범위 {1} 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteMissileTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteSniperTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">획득하는 골드 {0}/{1} % 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">projectile_prefab_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stage_inspection_time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0}/{1} % 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MissileProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ColdAirProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SniperProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10004;10005;10006;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MissileTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">replace_train_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10001;10002;10003;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염으로 지속적인 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NormalTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SniperTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CannonProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격 딜레이 {0}/{1} % 감소</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NormalProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LaserTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExplosionRangeTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">weighted_upgrades</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_upgrade_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExplosionProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ColdAirRangeTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CannonTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElectrickProjectile</t>
+    <t xml:space="preserve">적 처치 시 획득하는 골드가 {0}({1})만큼 증가합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">적 처치 시 획득하는 경험치가 {0}({1})만큼 증가합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">need_money</t>
+  </si>
+  <si>
+    <t xml:space="preserve">move_speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레이저 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고블린 창병이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 냉기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 화염 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SkullKing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1;1;1;1;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전기 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 전기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GoblinSpear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stat_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 저격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MainTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 레이저 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 폭발 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prefab_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포격 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GiantGoblin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고블린 주술사다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">폭발 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">train_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 포격 포탑</t>
   </si>
   <si>
     <t xml:space="preserve">description</t>
   </si>
   <si>
-    <t xml:space="preserve">저격 포탑 강화</t>
+    <t xml:space="preserve">냉기 포탑 강화</t>
   </si>
   <si>
     <t xml:space="preserve">엘리트 기관총 포탑</t>
   </si>
   <si>
-    <t xml:space="preserve">공격력 {0} 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">train_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폭발 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 전기 포탑</t>
+    <t xml:space="preserve">Minotaur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 미사일 포탑</t>
   </si>
   <si>
     <t xml:space="preserve">Hammershark</t>
   </si>
   <si>
-    <t xml:space="preserve">GiantGoblin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 폭발 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MainTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고블린 주술사다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">냉기 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minotaur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SkullKing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prefab_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 포격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 미사일 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 냉기 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">move_speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stat_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GoblinSpear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 레이저 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">need_money</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1;1;1;1;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 저격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고블린 창병이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 화염 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포탑들의 공격 딜레이가 {0}({1})만큼 감소합니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거대한 미사일을 발사해 몇 초 후 광역 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">범위 내에 있는 적들의 이동속도가 느려지고 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">적 처치 시 획득하는 경험치가 {0}({1})만큼 증가합니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">적 처치 시 획득하는 골드가 {0}({1})만큼 증가합니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_money_min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonTrainUpgrade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">target_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">체력 {0}/{1} % 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총으로 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TrainUpgrade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_exp_min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AttackDamage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GoblinSorcerer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AttackInterval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폭발 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">train_data_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">제일 기본이 되는 기차이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LaserProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_delay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FireTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_exp_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spawn_monsters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">냉기 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_damage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_money_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">target_train_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stage_end_time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">is_main_train</t>
-  </si>
-  <si>
-    <t xml:space="preserve">monster_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_interval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spawn_interval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑에 강화 버전이다.</t>
+    <t xml:space="preserve">1;5;5;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spawn_monsters_probability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포탑들의 공격력이 {0}({1})만큼 증가합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteExplosionRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격을 발사해 몇 초 후 강한 피해를 준다.</t>
   </si>
   <si>
     <t xml:space="preserve">10007;10008;10009;10010;</t>
   </si>
   <si>
-    <t xml:space="preserve">포탑들의 공격력이 {0}({1})만큼 증가합니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteExplosionRangeTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격을 발사해 몇 초 후 강한 피해를 준다.</t>
+    <t xml:space="preserve">포탑들의 체력이 {0}({1})만큼 증가합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 공격하는 적 수 {1} 증가</t>
   </si>
   <si>
     <t xml:space="preserve">범위 내에 있는 적들을 밀치고 피해를 준다.</t>
@@ -544,19 +556,10 @@
     <t xml:space="preserve">미사일로 강한 피해를 준다. 공격속도는 느리다.</t>
   </si>
   <si>
-    <t xml:space="preserve">spawn_monsters_probability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 공격하는 적 수 {1} 증가</t>
+    <t xml:space="preserve">EliteElectrickTurretTrain</t>
   </si>
   <si>
     <t xml:space="preserve">화면에 있는 다수의 적들을 전기로 공격한다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포탑들의 체력이 {0}({1})만큼 증가합니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteElectrickTurretTrain</t>
   </si>
 </sst>
 </file>
@@ -945,31 +948,7 @@
   <cellStyles count="1">
     <cellStyle xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAE3F3"/>
-          <bgColor rgb="FFDAE3F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAE3F3"/>
-          <bgColor rgb="FFDAE3F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1071,13 +1050,10 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="1" count="1">
-      <tableStyleElement type="headerRow" size="1" dxfId="4"/>
+      <tableStyleElement type="headerRow" size="1" dxfId="1"/>
     </tableStyle>
-    <tableStyle name="Light Style 1 - Accent 1" pivot="0" table="1" count="4">
-      <tableStyleElement type="wholeTable" size="1" dxfId="3"/>
-      <tableStyleElement type="headerRow" size="1" dxfId="2"/>
-      <tableStyleElement type="totalRow" size="1" dxfId="1"/>
-      <tableStyleElement type="firstColumn" size="1"/>
+    <tableStyle name="Light Style 1 - Accent 1" pivot="0" table="1" count="1">
+      <tableStyleElement type="wholeTable" size="1"/>
     </tableStyle>
   </tableStyles>
 </styleSheet>
@@ -1394,46 +1370,46 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>162</v>
+        <v>66</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>91</v>
+        <v>161</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>151</v>
+        <v>61</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>140</v>
+        <v>63</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>153</v>
+        <v>83</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>131</v>
+        <v>73</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>157</v>
+        <v>76</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>159</v>
+        <v>67</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>117</v>
+        <v>145</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -1441,10 +1417,10 @@
         <v>10001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>4</v>
+        <v>93</v>
       </c>
       <c r="D2" s="7">
         <v>10</v>
@@ -1456,16 +1432,16 @@
         <v>5</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="I2" s="7">
         <v>10</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="K2" s="7">
         <v>10</v>
@@ -1474,10 +1450,10 @@
         <v>2</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -1485,10 +1461,10 @@
         <v>10002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>10</v>
+        <v>109</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
       <c r="D3" s="5">
         <v>35</v>
@@ -1518,10 +1494,10 @@
         <v>1.5</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>10</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -1529,10 +1505,10 @@
         <v>10003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>31</v>
+        <v>118</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>21</v>
+        <v>106</v>
       </c>
       <c r="D4" s="5">
         <v>50</v>
@@ -1562,10 +1538,10 @@
         <v>6</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>31</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -1573,10 +1549,10 @@
         <v>10004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>99</v>
+        <v>166</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="D5" s="5">
         <v>60</v>
@@ -1606,10 +1582,10 @@
         <v>2</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>99</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -1617,10 +1593,10 @@
         <v>10005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>26</v>
+        <v>113</v>
       </c>
       <c r="D6" s="5">
         <v>40</v>
@@ -1650,10 +1626,10 @@
         <v>5</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>19</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -1661,10 +1637,10 @@
         <v>10006</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>20</v>
+        <v>107</v>
       </c>
       <c r="D7" s="5">
         <v>200</v>
@@ -1694,10 +1670,10 @@
         <v>2</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -1705,10 +1681,10 @@
         <v>10007</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>35</v>
+        <v>116</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="D8" s="5">
         <v>40</v>
@@ -1738,10 +1714,10 @@
         <v>3</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>35</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -1749,10 +1725,10 @@
         <v>10008</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>16</v>
+        <v>98</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="D9" s="5">
         <v>70</v>
@@ -1782,10 +1758,10 @@
         <v>1.5</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>16</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -1793,10 +1769,10 @@
         <v>10009</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>14</v>
+        <v>108</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>18</v>
+        <v>111</v>
       </c>
       <c r="D10" s="5">
         <v>100</v>
@@ -1826,10 +1802,10 @@
         <v>1.5</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>14</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -1837,10 +1813,10 @@
         <v>10010</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>36</v>
+        <v>121</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="D11" s="5">
         <v>150</v>
@@ -1870,10 +1846,10 @@
         <v>2</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>36</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -1881,10 +1857,10 @@
         <v>10011</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>8</v>
+        <v>95</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>30</v>
+        <v>112</v>
       </c>
       <c r="D12" s="5">
         <v>30</v>
@@ -1914,10 +1890,10 @@
         <v>2</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>8</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -1925,10 +1901,10 @@
         <v>10012</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>32</v>
+        <v>129</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="D13" s="5">
         <v>100</v>
@@ -1958,10 +1934,10 @@
         <v>3</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>32</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -1969,10 +1945,10 @@
         <v>10013</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>107</v>
+        <v>164</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="D14" s="5">
         <v>250</v>
@@ -2002,10 +1978,10 @@
         <v>2</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>107</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -2013,10 +1989,10 @@
         <v>10014</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="D15" s="5">
         <v>60</v>
@@ -2046,10 +2022,10 @@
         <v>2</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -2057,10 +2033,10 @@
         <v>10015</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>142</v>
+        <v>65</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>104</v>
+        <v>155</v>
       </c>
       <c r="D16" s="5">
         <v>60</v>
@@ -2090,10 +2066,10 @@
         <v>5</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>142</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -2101,10 +2077,10 @@
         <v>10016</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>100</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>17</v>
       </c>
       <c r="D17" s="5">
         <v>300</v>
@@ -2134,10 +2110,10 @@
         <v>2</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>100</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -2145,10 +2121,10 @@
         <v>10100</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>108</v>
+        <v>139</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>11</v>
+        <v>123</v>
       </c>
       <c r="D22" s="5">
         <v>500</v>
@@ -2178,10 +2154,10 @@
         <v>3</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>108</v>
+        <v>139</v>
       </c>
       <c r="O22" s="2"/>
     </row>
@@ -2205,31 +2181,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>135</v>
+        <v>57</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>91</v>
+        <v>161</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>159</v>
+        <v>67</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>156</v>
+        <v>84</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>132</v>
+        <v>81</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>163</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -2237,10 +2213,10 @@
         <v>100001</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>96</v>
+        <v>158</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F2" s="7">
         <v>1</v>
@@ -2254,10 +2230,10 @@
         <v>100001</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>96</v>
+        <v>158</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F3" s="7">
         <v>1</v>
@@ -2271,10 +2247,10 @@
         <v>100001</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>96</v>
+        <v>158</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F4" s="7">
         <v>1</v>
@@ -2288,10 +2264,10 @@
         <v>100002</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>106</v>
+        <v>162</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F5" s="7">
         <v>1</v>
@@ -2306,10 +2282,10 @@
         <v>100002</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>106</v>
+        <v>162</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F6" s="7">
         <v>1</v>
@@ -2323,10 +2299,10 @@
         <v>100002</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>106</v>
+        <v>162</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F7" s="7">
         <v>1</v>
@@ -2359,31 +2335,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>135</v>
+        <v>57</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>91</v>
+        <v>161</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>146</v>
+        <v>51</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>86</v>
+        <v>27</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>147</v>
+        <v>53</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>115</v>
+        <v>144</v>
       </c>
       <c r="J1" s="8"/>
     </row>
@@ -2392,10 +2368,10 @@
         <v>110001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2407,10 +2383,10 @@
         <v>100</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>139</v>
+        <v>68</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>141</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2418,10 +2394,10 @@
         <v>110002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>80</v>
+        <v>44</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
       <c r="D3" s="7">
         <v>200</v>
@@ -2433,10 +2409,10 @@
         <v>100</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>139</v>
+        <v>68</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>143</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2444,10 +2420,10 @@
         <v>110003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>136</v>
+        <v>54</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D4" s="7">
         <v>50</v>
@@ -2459,10 +2435,10 @@
         <v>50</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>139</v>
+        <v>68</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>22</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2470,7 +2446,7 @@
         <v>110004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>63</v>
+        <v>14</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>130</v>
@@ -2485,7 +2461,7 @@
         <v>10</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>133</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2493,10 +2469,10 @@
         <v>110005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D6" s="7">
         <v>500</v>
@@ -2508,7 +2484,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>133</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -2530,25 +2506,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>95</v>
+        <v>159</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>91</v>
+        <v>161</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>161</v>
+        <v>70</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2556,10 +2532,10 @@
         <v>20001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>37</v>
+        <v>89</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>149</v>
+        <v>82</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2568,7 +2544,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>103</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2595,40 +2571,40 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>95</v>
+        <v>159</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>91</v>
+        <v>161</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>161</v>
+        <v>70</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>159</v>
+        <v>67</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>156</v>
+        <v>84</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>132</v>
+        <v>81</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>163</v>
+        <v>78</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>64</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2636,10 +2612,10 @@
         <v>40001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2648,7 +2624,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>84</v>
+        <v>37</v>
       </c>
       <c r="H2" s="7">
         <v>5</v>
@@ -2663,7 +2639,7 @@
         <v>4</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>87</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -2671,10 +2647,10 @@
         <v>40002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>33</v>
+        <v>119</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>128</v>
+        <v>87</v>
       </c>
       <c r="D3" s="7">
         <v>100</v>
@@ -2683,7 +2659,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>88</v>
+        <v>45</v>
       </c>
       <c r="H3" s="7">
         <v>5</v>
@@ -2698,7 +2674,7 @@
         <v>0.10000000000000001</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:1">
@@ -2716,10 +2692,10 @@
         <v>41001</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>102</v>
+        <v>149</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>145</v>
+        <v>50</v>
       </c>
       <c r="D7" s="7">
         <v>150</v>
@@ -2728,7 +2704,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H7" s="7">
         <v>8</v>
@@ -2743,7 +2719,7 @@
         <v>4</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>87</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2751,10 +2727,10 @@
         <v>41002</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>155</v>
+        <v>69</v>
       </c>
       <c r="D8" s="7">
         <v>150</v>
@@ -2763,7 +2739,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="H8" s="7">
         <v>13</v>
@@ -2778,7 +2754,7 @@
         <v>0.10000000000000001</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2807,7 +2783,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:N21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
   <cols>
     <col min="1" max="1" width="15.640625" style="7" customWidth="1"/>
     <col min="2" max="2" width="17.640625" style="7" customWidth="1"/>
@@ -2821,54 +2797,54 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>95</v>
+        <v>159</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>91</v>
+        <v>161</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>161</v>
+        <v>70</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>159</v>
+        <v>67</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>156</v>
+        <v>84</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>132</v>
+        <v>81</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>163</v>
+        <v>78</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>134</v>
+        <v>56</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="16.75">
       <c r="A2" s="9">
         <v>30001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>34</v>
+        <v>122</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>138</v>
+        <v>55</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2877,7 +2853,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="H2" s="7">
         <v>10</v>
@@ -2895,7 +2871,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="8" t="s">
-        <v>81</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2903,10 +2879,10 @@
         <v>30002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>27</v>
+        <v>124</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>75</v>
+        <v>39</v>
       </c>
       <c r="D3" s="7">
         <v>100</v>
@@ -2915,7 +2891,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>152</v>
+        <v>64</v>
       </c>
       <c r="H3" s="7">
         <v>10</v>
@@ -2933,7 +2909,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>49</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2941,10 +2917,10 @@
         <v>30003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>23</v>
+        <v>114</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="D4" s="7">
         <v>100</v>
@@ -2953,7 +2929,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H4" s="7">
         <v>10</v>
@@ -2971,7 +2947,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>67</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -2979,10 +2955,10 @@
         <v>30004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>7</v>
+        <v>91</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>51</v>
+        <v>8</v>
       </c>
       <c r="D5" s="7">
         <v>100</v>
@@ -2991,7 +2967,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>82</v>
+        <v>36</v>
       </c>
       <c r="H5" s="7">
         <v>15</v>
@@ -3009,7 +2985,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>150</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3017,10 +2993,10 @@
         <v>30005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>9</v>
+        <v>97</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D6" s="7">
         <v>100</v>
@@ -3029,7 +3005,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="H6" s="7">
         <v>10</v>
@@ -3047,7 +3023,7 @@
         <v>5</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>90</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3055,10 +3031,10 @@
         <v>30006</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>13</v>
+        <v>102</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>127</v>
+        <v>88</v>
       </c>
       <c r="D7" s="7">
         <v>100</v>
@@ -3067,7 +3043,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>89</v>
+        <v>26</v>
       </c>
       <c r="H7" s="7">
         <v>10</v>
@@ -3085,7 +3061,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -3093,10 +3069,10 @@
         <v>30007</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>24</v>
+        <v>110</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D8" s="7">
         <v>100</v>
@@ -3105,7 +3081,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
       <c r="H8" s="7">
         <v>10</v>
@@ -3123,7 +3099,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:1">
@@ -3135,15 +3111,15 @@
     <row r="11" spans="1:1">
       <c r="A11" s="10"/>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" ht="16.75">
       <c r="A12" s="11">
         <v>31001</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>93</v>
+        <v>163</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="D12" s="7">
         <v>150</v>
@@ -3152,7 +3128,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="H12" s="1">
         <v>10</v>
@@ -3170,7 +3146,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="8" t="s">
-        <v>81</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -3178,10 +3154,10 @@
         <v>31002</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>137</v>
+        <v>79</v>
       </c>
       <c r="D13" s="7">
         <v>150</v>
@@ -3190,7 +3166,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="H13" s="7">
         <v>10</v>
@@ -3208,18 +3184,18 @@
         <v>0</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="16.75">
       <c r="A14" s="11">
         <v>31003</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>112</v>
+        <v>165</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>83</v>
+        <v>35</v>
       </c>
       <c r="D14" s="7">
         <v>150</v>
@@ -3228,7 +3204,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="H14" s="7">
         <v>10</v>
@@ -3246,7 +3222,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>67</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -3254,10 +3230,10 @@
         <v>31004</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>71</v>
+        <v>43</v>
       </c>
       <c r="D15" s="7">
         <v>150</v>
@@ -3266,7 +3242,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="H15" s="7">
         <v>10</v>
@@ -3284,18 +3260,18 @@
         <v>0</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="16.75">
       <c r="A16" s="11">
         <v>31005</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>98</v>
+        <v>142</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>166</v>
+        <v>60</v>
       </c>
       <c r="D16" s="7">
         <v>150</v>
@@ -3322,7 +3298,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>90</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -3330,10 +3306,10 @@
         <v>31006</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>111</v>
+        <v>160</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>144</v>
+        <v>58</v>
       </c>
       <c r="D17" s="7">
         <v>150</v>
@@ -3342,7 +3318,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="H17" s="7">
         <v>10</v>
@@ -3360,18 +3336,18 @@
         <v>0</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="16.75">
       <c r="A18" s="11">
         <v>31007</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>164</v>
+        <v>71</v>
       </c>
       <c r="D18" s="7">
         <v>150</v>
@@ -3380,7 +3356,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="H18" s="7">
         <v>10</v>
@@ -3398,7 +3374,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -3407,7 +3383,7 @@
     <row r="20" spans="1:1">
       <c r="A20" s="12"/>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" ht="16.75">
       <c r="A21" s="13"/>
     </row>
   </sheetData>
@@ -3433,25 +3409,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>165</v>
+        <v>85</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>154</v>
+        <v>75</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3468,13 +3444,13 @@
         <v>0.5</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>5</v>
+        <v>96</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>5</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -3491,13 +3467,13 @@
         <v>0.5</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>5</v>
+        <v>96</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>5</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -3514,13 +3490,13 @@
         <v>0.5</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -3545,19 +3521,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>148</v>
+        <v>80</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="16.75">
@@ -3596,7 +3572,7 @@
         <v>30003</v>
       </c>
       <c r="C4" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="19">
         <v>0</v>
@@ -3624,7 +3600,7 @@
         <v>30005</v>
       </c>
       <c r="C6" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="19">
         <v>0</v>
@@ -3757,19 +3733,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>158</v>
+        <v>77</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>0</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.75">
@@ -3968,7 +3944,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
   <cols>
     <col min="1" max="1" width="15.78515625" style="7" customWidth="1"/>
     <col min="2" max="2" width="13.5" style="7" customWidth="1"/>
@@ -3976,19 +3952,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>135</v>
+        <v>57</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>91</v>
+        <v>161</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -4006,7 +3982,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:J22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.4"/>
   <cols>
     <col min="2" max="2" width="17.28515625" style="7" customWidth="1"/>
     <col min="3" max="3" width="35.0703125" style="7" customWidth="1"/>
@@ -4020,31 +3996,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>135</v>
+        <v>57</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>91</v>
+        <v>161</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>159</v>
+        <v>67</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>156</v>
+        <v>84</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>132</v>
+        <v>81</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>163</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -4052,10 +4028,10 @@
         <v>90001</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>97</v>
+        <v>153</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="G2" s="7">
         <v>5</v>
@@ -4069,10 +4045,10 @@
         <v>90001</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>97</v>
+        <v>153</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="G3" s="7">
         <v>10</v>
@@ -4086,10 +4062,10 @@
         <v>90001</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>97</v>
+        <v>153</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="G4" s="7">
         <v>25</v>
@@ -4103,10 +4079,10 @@
         <v>90002</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="G5" s="7">
         <v>2</v>
@@ -4117,10 +4093,10 @@
         <v>90002</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="G6" s="7">
         <v>5</v>
@@ -4131,10 +4107,10 @@
         <v>90002</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="G7" s="7">
         <v>10</v>
@@ -4145,10 +4121,10 @@
         <v>90003</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>105</v>
+        <v>157</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="G8" s="7">
         <v>15</v>
@@ -4162,10 +4138,10 @@
         <v>90003</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>105</v>
+        <v>157</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="G9" s="7">
         <v>20</v>
@@ -4179,10 +4155,10 @@
         <v>90003</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>105</v>
+        <v>157</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="G10" s="7">
         <v>40</v>
@@ -4196,10 +4172,10 @@
         <v>90004</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="G11" s="7">
         <v>50</v>
@@ -4210,10 +4186,10 @@
         <v>90004</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="G12" s="7">
         <v>150</v>
@@ -4224,10 +4200,10 @@
         <v>90004</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="G13" s="7">
         <v>250</v>
@@ -4238,7 +4214,7 @@
         <v>90005</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>101</v>
+        <v>141</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>174</v>
@@ -4255,7 +4231,7 @@
         <v>90005</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>101</v>
+        <v>141</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>174</v>
@@ -4272,7 +4248,7 @@
         <v>90005</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>101</v>
+        <v>141</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>174</v>
@@ -4289,10 +4265,10 @@
         <v>90006</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>109</v>
+        <v>151</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="F17" s="7">
         <v>1</v>
@@ -4306,10 +4282,10 @@
         <v>90006</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>109</v>
+        <v>151</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="F18" s="7">
         <v>1</v>
@@ -4323,10 +4299,10 @@
         <v>90006</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>109</v>
+        <v>151</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="F19" s="7">
         <v>1</v>
@@ -4340,10 +4316,10 @@
         <v>90007</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>92</v>
+        <v>156</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="G20" s="7">
         <v>50</v>
@@ -4354,10 +4330,10 @@
         <v>90007</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>92</v>
+        <v>156</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="G21" s="7">
         <v>150</v>
@@ -4368,10 +4344,10 @@
         <v>90007</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>92</v>
+        <v>156</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="G22" s="7">
         <v>350</v>

</xml_diff>

<commit_message>
fix : CannonProjectile 이미지 변경, Cannon 공격 방식 변경
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/TrainDefenseData.xlsx
+++ b/Assets/02_Resources/Data/TrainDefenseData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.4575"/>
   <workbookPr codeName="ThisWorkbook" autoCompressPictures="1"/>
   <bookViews>
-    <workbookView windowWidth="28545" windowHeight="11700" tabRatio="839" activeTab="4"/>
+    <workbookView windowWidth="28545" windowHeight="11700" tabRatio="839" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Monster_Data" sheetId="1" r:id="rId4"/>
@@ -23,60 +23,171 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="179">
+  <si>
+    <t xml:space="preserve">AttackInterval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전기 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_exp_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_delay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">monster_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FireTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">체력 {0}/{1} % 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GoblinSorcerer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">폭발 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonTrainUpgrade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총으로 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포격 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AttackDamage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">train_data_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_money_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">제일 기본이 되는 기차이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_damage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spawn_interval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_main_train</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_interval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stage_end_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target_train_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LaserProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_exp_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_money_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">냉기 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spawn_monsters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TrainUpgrade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteColdAirRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 공격 범위 {1} 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteMissileTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteSniperTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteNormalTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">획득하는 경험치 {0}/{1} % 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteLaserTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteFireTurretTrain</t>
+  </si>
   <si>
     <t xml:space="preserve">spawn_monsters_level</t>
   </si>
   <si>
+    <t xml:space="preserve">레이저로 강하게 지속적인 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 공격딜레이 {1} 감소</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteCannonTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FireEffectProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stage_inspection_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElectrickTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">projectile_prefab_id</t>
+  </si>
+  <si>
     <t xml:space="preserve">공격력 {0} 증가 범위 {1} 증가</t>
   </si>
   <si>
-    <t xml:space="preserve">획득하는 경험치 {0}/{1} % 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FireEffectProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteCannonTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteLaserTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 공격딜레이 {1} 감소</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteSniperTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저로 강하게 지속적인 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">projectile_prefab_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteMissileTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stage_inspection_time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteNormalTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 공격 범위 {1} 증가</t>
-  </si>
-  <si>
     <t xml:space="preserve">획득하는 골드 {0}/{1} % 증가</t>
   </si>
   <si>
-    <t xml:space="preserve">EliteFireTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteColdAirRangeTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElectrickTurretTrain</t>
+    <t xml:space="preserve">10</t>
   </si>
   <si>
     <t xml:space="preserve">곰이다</t>
@@ -85,346 +196,250 @@
     <t xml:space="preserve">거미다</t>
   </si>
   <si>
+    <t xml:space="preserve">판다다</t>
+  </si>
+  <si>
     <t xml:space="preserve">뱀이다</t>
   </si>
   <si>
+    <t xml:space="preserve">id</t>
+  </si>
+  <si>
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">판다다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id</t>
+    <t xml:space="preserve">적 처치 시 획득하는 골드가 {0}({1})만큼 증가합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">적 처치 시 획득하는 경험치가 {0}({1})만큼 증가합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LaserTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10001;10002;10003;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_upgrade_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CannonProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격 딜레이 {0}/{1} % 감소</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레이저 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염으로 지속적인 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElectrickProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SniperTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExplosionRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MissileTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weighted_upgrades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ColdAirRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NormalTurretTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SniperProjectile</t>
   </si>
   <si>
     <t xml:space="preserve">10004;10005;10006;</t>
   </si>
   <si>
+    <t xml:space="preserve">ColdAirProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">replace_train_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NormalProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일 포탑에 강화 버전이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MissileProjectile</t>
+  </si>
+  <si>
     <t xml:space="preserve">CannonTurretTrain</t>
   </si>
   <si>
-    <t xml:space="preserve">max_upgrade_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElectrickProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SniperTurretTrain</t>
-  </si>
-  <si>
     <t xml:space="preserve">ExplosionProjectile</t>
   </si>
   <si>
-    <t xml:space="preserve">weighted_upgrades</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MissileProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ColdAirProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LaserTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExplosionRangeTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NormalProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염으로 지속적인 피해를 준다.</t>
-  </si>
-  <si>
     <t xml:space="preserve">공격력 {0}/{1} % 증가</t>
   </si>
   <si>
-    <t xml:space="preserve">CannonProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10001;10002;10003;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격 딜레이 {0}/{1} % 감소</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ColdAirRangeTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MissileTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SniperProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NormalTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">replace_train_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폭발 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NonTrainUpgrade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">체력 {0}/{1} % 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총으로 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">target_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AttackDamage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_delay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AttackInterval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_exp_min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FireTurretTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GoblinSorcerer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">monster_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TrainUpgrade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">냉기 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">is_main_train</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stage_end_time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_money_min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LaserProjectile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spawn_monsters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_money_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">target_train_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_interval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염 포탑에 강화 버전이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">train_data_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">제일 기본이 되는 기차이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop_exp_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_damage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spawn_interval</t>
+    <t xml:space="preserve">damage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">도적이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미노타우로스다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레이저 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1;1;1;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">해골 병사다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">메인 기차</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dwarf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고블린 거인</t>
+  </si>
+  <si>
+    <t xml:space="preserve">놀이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관총 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">도마뱀이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">냉기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">상어다 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거북이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ranged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_hp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">해골 왕이당.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">icon_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">귀상어다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spider</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1;5;5;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skull</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gnoll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화염 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lizard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turtle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">폭발 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxHp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">난쟁이다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">범위 내에 있는 적들의 이동속도가 느려지고 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거대한 미사일을 발사해 몇 초 후 광역 피해를 준다.</t>
   </si>
   <si>
     <t xml:space="preserve">포탑들의 공격 딜레이가 {0}({1})만큼 감소합니다.</t>
   </si>
   <si>
-    <t xml:space="preserve">범위 내에 있는 적들의 이동속도가 느려지고 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거대한 미사일을 발사해 몇 초 후 광역 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">메인 기차</t>
-  </si>
-  <si>
-    <t xml:space="preserve">도적이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">damage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">해골 병사다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미노타우로스다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dwarf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1;1;1;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고블린 거인</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxHp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폭발 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Turtle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">놀이다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거북이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lizard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thief</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">도마뱀이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">난쟁이다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">상어다 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skull</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Snake</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gnoll</t>
-  </si>
-  <si>
-    <t xml:space="preserve">냉기 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Melee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">해골 왕이당.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ranged</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_hp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">icon_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">귀상어다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spider</t>
-  </si>
-  <si>
-    <t xml:space="preserve">적 처치 시 획득하는 골드가 {0}({1})만큼 증가합니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">적 처치 시 획득하는 경험치가 {0}({1})만큼 증가합니다.</t>
+    <t xml:space="preserve">move_speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 냉기 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SkullKing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1;1;1;1;</t>
   </si>
   <si>
     <t xml:space="preserve">need_money</t>
   </si>
   <si>
-    <t xml:space="preserve">move_speed</t>
+    <t xml:space="preserve">전기 포탑 강화</t>
   </si>
   <si>
     <t xml:space="preserve">레이저 포탑 강화</t>
@@ -433,130 +448,115 @@
     <t xml:space="preserve">고블린 창병이다</t>
   </si>
   <si>
-    <t xml:space="preserve">엘리트 냉기 포탑</t>
-  </si>
-  <si>
     <t xml:space="preserve">엘리트 화염 포탑</t>
   </si>
   <si>
     <t xml:space="preserve">화염 포탑 강화</t>
   </si>
   <si>
-    <t xml:space="preserve">SkullKing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1;1;1;1;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑 강화</t>
+    <t xml:space="preserve">GoblinSpear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고블린 주술사다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저격 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 레이저 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엘리트 폭발 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MainTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attack_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일 포탑 강화</t>
   </si>
   <si>
     <t xml:space="preserve">엘리트 전기 포탑</t>
   </si>
   <si>
-    <t xml:space="preserve">GoblinSpear</t>
-  </si>
-  <si>
     <t xml:space="preserve">stat_type</t>
   </si>
   <si>
-    <t xml:space="preserve">attack_type</t>
+    <t xml:space="preserve">prefab_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포격 포탑 강화</t>
   </si>
   <si>
     <t xml:space="preserve">엘리트 저격 포탑</t>
   </si>
   <si>
-    <t xml:space="preserve">MainTrain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 레이저 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 폭발 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prefab_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가</t>
-  </si>
-  <si>
     <t xml:space="preserve">기관총 포탑 강화</t>
   </si>
   <si>
     <t xml:space="preserve">GiantGoblin</t>
   </si>
   <si>
-    <t xml:space="preserve">고블린 주술사다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑 강화</t>
+    <t xml:space="preserve">냉기 포탑 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
   </si>
   <si>
     <t xml:space="preserve">폭발 포탑 강화</t>
   </si>
   <si>
+    <t xml:space="preserve">엘리트 포격 포탑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minotaur</t>
+  </si>
+  <si>
     <t xml:space="preserve">train_name</t>
   </si>
   <si>
-    <t xml:space="preserve">엘리트 포격 포탑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">냉기 포탑 강화</t>
+    <t xml:space="preserve">엘리트 미사일 포탑</t>
   </si>
   <si>
     <t xml:space="preserve">엘리트 기관총 포탑</t>
   </si>
   <si>
-    <t xml:space="preserve">Minotaur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엘리트 미사일 포탑</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hammershark</t>
   </si>
   <si>
-    <t xml:space="preserve">1;5;5;</t>
-  </si>
-  <si>
     <t xml:space="preserve">spawn_monsters_probability</t>
   </si>
   <si>
+    <t xml:space="preserve">10007;10008;10009;10010;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">포탑들의 체력이 {0}({1})만큼 증가합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteExplosionRangeTrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공격력 {0} 증가 공격하는 적 수 {1} 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">범위 내에 있는 적들을 밀치고 피해를 준다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미사일로 강한 피해를 준다. 공격속도는 느리다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EliteElectrickTurretTrain</t>
+  </si>
+  <si>
     <t xml:space="preserve">포탑들의 공격력이 {0}({1})만큼 증가합니다.</t>
   </si>
   <si>
-    <t xml:space="preserve">EliteExplosionRangeTrain</t>
-  </si>
-  <si>
     <t xml:space="preserve">저격을 발사해 몇 초 후 강한 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10007;10008;10009;10010;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포탑들의 체력이 {0}({1})만큼 증가합니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 {0} 증가 공격하는 적 수 {1} 증가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">범위 내에 있는 적들을 밀치고 피해를 준다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일로 강한 피해를 준다. 공격속도는 느리다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EliteElectrickTurretTrain</t>
   </si>
   <si>
     <t xml:space="preserve">화면에 있는 다수의 적들을 전기로 공격한다.</t>
@@ -948,15 +948,7 @@
   <cellStyles count="1">
     <cellStyle xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1050,11 +1042,9 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="1" count="1">
-      <tableStyleElement type="headerRow" size="1" dxfId="1"/>
+      <tableStyleElement type="headerRow" size="1"/>
     </tableStyle>
-    <tableStyle name="Light Style 1 - Accent 1" pivot="0" table="1" count="1">
-      <tableStyleElement type="wholeTable" size="1"/>
-    </tableStyle>
+    <tableStyle name="Light Style 1 - Accent 1" pivot="0" table="1"/>
   </tableStyles>
 </styleSheet>
 </file>
@@ -1370,46 +1360,46 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>66</v>
+        <v>4</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>133</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>76</v>
+        <v>18</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -1417,7 +1407,7 @@
         <v>10001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>93</v>
@@ -1432,16 +1422,16 @@
         <v>5</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="I2" s="7">
         <v>10</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="K2" s="7">
         <v>10</v>
@@ -1450,10 +1440,10 @@
         <v>2</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -1461,10 +1451,10 @@
         <v>10002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D3" s="5">
         <v>35</v>
@@ -1494,10 +1484,10 @@
         <v>1.5</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -1505,10 +1495,10 @@
         <v>10003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D4" s="5">
         <v>50</v>
@@ -1538,10 +1528,10 @@
         <v>6</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -1549,10 +1539,10 @@
         <v>10004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="D5" s="5">
         <v>60</v>
@@ -1582,10 +1572,10 @@
         <v>2</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -1593,10 +1583,10 @@
         <v>10005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D6" s="5">
         <v>40</v>
@@ -1626,10 +1616,10 @@
         <v>5</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -1637,7 +1627,7 @@
         <v>10006</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>107</v>
@@ -1670,10 +1660,10 @@
         <v>2</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -1681,10 +1671,10 @@
         <v>10007</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="D8" s="5">
         <v>40</v>
@@ -1714,10 +1704,10 @@
         <v>3</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -1725,10 +1715,10 @@
         <v>10008</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="D9" s="5">
         <v>70</v>
@@ -1758,10 +1748,10 @@
         <v>1.5</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -1769,10 +1759,10 @@
         <v>10009</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="D10" s="5">
         <v>100</v>
@@ -1802,10 +1792,10 @@
         <v>1.5</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -1813,10 +1803,10 @@
         <v>10010</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="D11" s="5">
         <v>150</v>
@@ -1846,10 +1836,10 @@
         <v>2</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -1857,10 +1847,10 @@
         <v>10011</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="D12" s="5">
         <v>30</v>
@@ -1890,10 +1880,10 @@
         <v>2</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -1901,10 +1891,10 @@
         <v>10012</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="D13" s="5">
         <v>100</v>
@@ -1934,10 +1924,10 @@
         <v>3</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -1945,10 +1935,10 @@
         <v>10013</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D14" s="5">
         <v>250</v>
@@ -1978,10 +1968,10 @@
         <v>2</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -1992,7 +1982,7 @@
         <v>143</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D15" s="5">
         <v>60</v>
@@ -2022,7 +2012,7 @@
         <v>2</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N15" s="2" t="s">
         <v>143</v>
@@ -2033,10 +2023,10 @@
         <v>10015</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="D16" s="5">
         <v>60</v>
@@ -2066,10 +2056,10 @@
         <v>5</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -2077,10 +2067,10 @@
         <v>10016</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D17" s="5">
         <v>300</v>
@@ -2110,10 +2100,10 @@
         <v>2</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -2121,10 +2111,10 @@
         <v>10100</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="D22" s="5">
         <v>500</v>
@@ -2154,10 +2144,10 @@
         <v>3</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="O22" s="2"/>
     </row>
@@ -2181,31 +2171,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>81</v>
+        <v>26</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>78</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -2213,10 +2203,10 @@
         <v>100001</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="F2" s="7">
         <v>1</v>
@@ -2230,10 +2220,10 @@
         <v>100001</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="F3" s="7">
         <v>1</v>
@@ -2247,10 +2237,10 @@
         <v>100001</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="F4" s="7">
         <v>1</v>
@@ -2264,10 +2254,10 @@
         <v>100002</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="F5" s="7">
         <v>1</v>
@@ -2282,10 +2272,10 @@
         <v>100002</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="F6" s="7">
         <v>1</v>
@@ -2299,10 +2289,10 @@
         <v>100002</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="F7" s="7">
         <v>1</v>
@@ -2335,31 +2325,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="J1" s="8"/>
     </row>
@@ -2368,10 +2358,10 @@
         <v>110001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>40</v>
+        <v>87</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2383,10 +2373,10 @@
         <v>100</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>59</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2394,10 +2384,10 @@
         <v>110002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>86</v>
+        <v>132</v>
       </c>
       <c r="D3" s="7">
         <v>200</v>
@@ -2409,10 +2399,10 @@
         <v>100</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2420,10 +2410,10 @@
         <v>110003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D4" s="7">
         <v>50</v>
@@ -2435,10 +2425,10 @@
         <v>50</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2446,10 +2436,10 @@
         <v>110004</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>14</v>
+        <v>53</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>130</v>
+        <v>61</v>
       </c>
       <c r="D5" s="7">
         <v>300</v>
@@ -2461,7 +2451,7 @@
         <v>10</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2469,10 +2459,10 @@
         <v>110005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>131</v>
+        <v>62</v>
       </c>
       <c r="D6" s="7">
         <v>500</v>
@@ -2484,7 +2474,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -2506,25 +2496,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>70</v>
+        <v>22</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2532,10 +2522,10 @@
         <v>20001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2544,7 +2534,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -2571,40 +2561,40 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>70</v>
+        <v>22</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>81</v>
+        <v>26</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>78</v>
+        <v>23</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2612,10 +2602,10 @@
         <v>40001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2624,7 +2614,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="H2" s="7">
         <v>5</v>
@@ -2639,7 +2629,7 @@
         <v>4</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>31</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -2647,10 +2637,10 @@
         <v>40002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>87</v>
+        <v>130</v>
       </c>
       <c r="D3" s="7">
         <v>100</v>
@@ -2659,7 +2649,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="H3" s="7">
         <v>5</v>
@@ -2674,7 +2664,7 @@
         <v>0.10000000000000001</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>34</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:1">
@@ -2692,10 +2682,10 @@
         <v>41001</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="D7" s="7">
         <v>150</v>
@@ -2704,7 +2694,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H7" s="7">
         <v>8</v>
@@ -2719,7 +2709,7 @@
         <v>4</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>31</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2727,10 +2717,10 @@
         <v>41002</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>69</v>
+        <v>32</v>
       </c>
       <c r="D8" s="7">
         <v>150</v>
@@ -2739,7 +2729,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="H8" s="7">
         <v>13</v>
@@ -2754,7 +2744,7 @@
         <v>0.10000000000000001</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>34</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2797,43 +2787,43 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>70</v>
+        <v>22</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>81</v>
+        <v>26</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>78</v>
+        <v>23</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="16.75">
@@ -2841,10 +2831,10 @@
         <v>30001</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="D2" s="7">
         <v>100</v>
@@ -2853,7 +2843,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="H2" s="7">
         <v>10</v>
@@ -2871,7 +2861,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="8" t="s">
-        <v>38</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2879,10 +2869,10 @@
         <v>30002</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="D3" s="7">
         <v>100</v>
@@ -2891,7 +2881,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>64</v>
+        <v>5</v>
       </c>
       <c r="H3" s="7">
         <v>10</v>
@@ -2909,7 +2899,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2917,10 +2907,10 @@
         <v>30003</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D4" s="7">
         <v>100</v>
@@ -2929,7 +2919,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="H4" s="7">
         <v>10</v>
@@ -2947,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -2958,7 +2948,7 @@
         <v>91</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="D5" s="7">
         <v>100</v>
@@ -2967,7 +2957,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="H5" s="7">
         <v>15</v>
@@ -2985,7 +2975,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>74</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2993,7 +2983,7 @@
         <v>30005</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>178</v>
@@ -3005,7 +2995,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="H6" s="7">
         <v>10</v>
@@ -3023,7 +3013,7 @@
         <v>5</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3031,10 +3021,10 @@
         <v>30006</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>88</v>
+        <v>131</v>
       </c>
       <c r="D7" s="7">
         <v>100</v>
@@ -3043,7 +3033,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>26</v>
+        <v>85</v>
       </c>
       <c r="H7" s="7">
         <v>10</v>
@@ -3061,7 +3051,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>41</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -3069,10 +3059,10 @@
         <v>30007</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D8" s="7">
         <v>100</v>
@@ -3081,7 +3071,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="H8" s="7">
         <v>10</v>
@@ -3099,7 +3089,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:1">
@@ -3116,10 +3106,10 @@
         <v>31001</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="D12" s="7">
         <v>150</v>
@@ -3128,7 +3118,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="H12" s="1">
         <v>10</v>
@@ -3146,7 +3136,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="8" t="s">
-        <v>38</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -3154,10 +3144,10 @@
         <v>31002</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="D13" s="7">
         <v>150</v>
@@ -3166,7 +3156,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="H13" s="7">
         <v>10</v>
@@ -3184,7 +3174,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="16.75">
@@ -3195,7 +3185,7 @@
         <v>165</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>35</v>
+        <v>83</v>
       </c>
       <c r="D14" s="7">
         <v>150</v>
@@ -3204,7 +3194,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="H14" s="7">
         <v>10</v>
@@ -3222,7 +3212,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -3230,10 +3220,10 @@
         <v>31004</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="D15" s="7">
         <v>150</v>
@@ -3242,7 +3232,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="H15" s="7">
         <v>10</v>
@@ -3260,7 +3250,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>74</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="16.75">
@@ -3268,10 +3258,10 @@
         <v>31005</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="D16" s="7">
         <v>150</v>
@@ -3280,7 +3270,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H16" s="7">
         <v>10</v>
@@ -3298,7 +3288,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -3306,10 +3296,10 @@
         <v>31006</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="D17" s="7">
         <v>150</v>
@@ -3318,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="H17" s="7">
         <v>10</v>
@@ -3336,7 +3326,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>41</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="16.75">
@@ -3344,10 +3334,10 @@
         <v>31007</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="D18" s="7">
         <v>150</v>
@@ -3356,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="H18" s="7">
         <v>10</v>
@@ -3374,7 +3364,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -3409,25 +3399,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>72</v>
-      </c>
       <c r="D1" s="25" t="s">
-        <v>85</v>
+        <v>21</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>168</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3444,13 +3434,13 @@
         <v>0.5</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>167</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -3467,13 +3457,13 @@
         <v>0.5</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -3490,13 +3480,13 @@
         <v>0.5</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -3521,19 +3511,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="16.75">
@@ -3572,7 +3562,7 @@
         <v>30003</v>
       </c>
       <c r="C4" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="19">
         <v>0</v>
@@ -3614,7 +3604,7 @@
         <v>30006</v>
       </c>
       <c r="C7" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="19">
         <v>0</v>
@@ -3733,19 +3723,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.75">
@@ -3952,19 +3942,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -3996,31 +3986,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="7" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>81</v>
+        <v>26</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>78</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -4028,10 +4018,10 @@
         <v>90001</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="G2" s="7">
         <v>5</v>
@@ -4045,10 +4035,10 @@
         <v>90001</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="G3" s="7">
         <v>10</v>
@@ -4062,10 +4052,10 @@
         <v>90001</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="G4" s="7">
         <v>25</v>
@@ -4079,10 +4069,10 @@
         <v>90002</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G5" s="7">
         <v>2</v>
@@ -4093,10 +4083,10 @@
         <v>90002</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G6" s="7">
         <v>5</v>
@@ -4107,10 +4097,10 @@
         <v>90002</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G7" s="7">
         <v>10</v>
@@ -4121,10 +4111,10 @@
         <v>90003</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="G8" s="7">
         <v>15</v>
@@ -4138,10 +4128,10 @@
         <v>90003</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="G9" s="7">
         <v>20</v>
@@ -4155,10 +4145,10 @@
         <v>90003</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="G10" s="7">
         <v>40</v>
@@ -4172,10 +4162,10 @@
         <v>90004</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G11" s="7">
         <v>50</v>
@@ -4186,10 +4176,10 @@
         <v>90004</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G12" s="7">
         <v>150</v>
@@ -4200,10 +4190,10 @@
         <v>90004</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G13" s="7">
         <v>250</v>
@@ -4214,10 +4204,10 @@
         <v>90005</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G14" s="7">
         <v>3</v>
@@ -4231,10 +4221,10 @@
         <v>90005</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G15" s="7">
         <v>5</v>
@@ -4248,10 +4238,10 @@
         <v>90005</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G16" s="7">
         <v>7</v>
@@ -4265,10 +4255,10 @@
         <v>90006</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F17" s="7">
         <v>1</v>
@@ -4282,10 +4272,10 @@
         <v>90006</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F18" s="7">
         <v>1</v>
@@ -4299,10 +4289,10 @@
         <v>90006</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F19" s="7">
         <v>1</v>
@@ -4316,10 +4306,10 @@
         <v>90007</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G20" s="7">
         <v>50</v>
@@ -4330,10 +4320,10 @@
         <v>90007</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G21" s="7">
         <v>150</v>
@@ -4344,10 +4334,10 @@
         <v>90007</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G22" s="7">
         <v>350</v>

</xml_diff>